<commit_message>
feat(ai): plan-analysis Edge Function + usePlanAI hook + sidebar gercek AI
- supabase/functions/plan-analysis/index.ts: Claude Haiku ile plan ozeti analizi
- src/modules/detailedplan/usePlanAI.ts: plan ID bazli cache, auto-trigger, refresh
- DetailedPlanShell.tsx: loading skeleton + insight listesi + action item

Deploy gerekiyor:
  npx supabase login
  npx supabase link --project-ref [proje-ref]
  npx supabase functions deploy plan-analysis --no-verify-jwt
  npx supabase secrets set ANTHROPIC_API_KEY=sk-ant-...

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/22.04.2026_masaustu_LDPE_Kömürcüler.xlsx
+++ b/22.04.2026_masaustu_LDPE_Kömürcüler.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48f45184d7e5c384/Desktop/Enba Similasyon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8637C44A-C109-4C22-ABBE-DDEB29A6CB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{8637C44A-C109-4C22-ABBE-DDEB29A6CB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DB67B33-9F59-4A9B-A220-4EDF54377E20}"/>
   <bookViews>
-    <workbookView xWindow="6480" yWindow="1176" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Değerler" sheetId="2" r:id="rId1"/>
@@ -1592,7 +1592,7 @@
         <v>12</v>
       </c>
       <c r="C6" s="3">
-        <f t="shared" ref="C4:C39" si="0">D6+E6</f>
+        <f t="shared" ref="C6:C7" si="0">D6+E6</f>
         <v>0</v>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
     <col min="8" max="8" width="6.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>1778.7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="16.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="16.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="25" t="s">
@@ -1991,7 +1991,7 @@
         <v>1778.7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="16.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="16.95" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="25" t="s">
@@ -2002,7 +2002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>1778.7</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -2051,7 +2051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" collapsed="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>1778.7</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>17</v>
       </c>
@@ -2088,7 +2088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="12" spans="1:6" collapsed="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>21</v>
       </c>
@@ -2114,7 +2114,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" collapsed="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>25</v>
       </c>
@@ -2170,7 +2170,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:4" hidden="1" outlineLevel="2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
       <c r="B17" s="7"/>
       <c r="C17" s="29" t="s">
@@ -2180,7 +2180,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:4" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>31</v>
       </c>
@@ -2299,7 +2299,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>47</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>49</v>
       </c>
@@ -2323,7 +2323,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
         <v>51</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>53</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>55</v>
       </c>
@@ -2359,7 +2359,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>57</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>59</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>61</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>63</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>64</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>3</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>66</v>
       </c>
@@ -2443,7 +2443,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>68</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:4" collapsed="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>70</v>
       </c>

</xml_diff>